<commit_message>
Walkthrough users workbooks of Cashiering, Product Maintenance and Renewal name the UAT site https://uat.brokerverse.cloud; Product Maintenance test cases with the UAT e-mail domain; User Access capture recipe for the grouped permission picker and the UAT e-mail domain
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_UAT_BRD-02_Business_Unit_Walkthrough_Users_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_UAT_BRD-02_Business_Unit_Walkthrough_Users_v1.0.xlsx
@@ -384,6 +384,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -409,6 +412,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -705,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B4:E31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -715,13 +721,16 @@
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="40" customHeight="1"/>
+    <row r="3"/>
     <row r="4" ht="6" customHeight="1">
       <c r="B4" s="1" t="n"/>
       <c r="C4" s="1" t="n"/>
       <c r="D4" s="1" t="n"/>
       <c r="E4" s="1" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -750,6 +759,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="B11" s="6" t="inlineStr">
         <is>
@@ -822,6 +832,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="9" t="inlineStr">
         <is>
@@ -867,7 +878,7 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>BIBS UAT environment (address issued with the passwords). Password: Issued separately by the iorta TechNXT Project Team</t>
+          <t>BIBS UAT environment: https://uat.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
         </is>
       </c>
       <c r="D21" s="14" t="n">
@@ -889,6 +900,7 @@
         <v>21</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="B24" s="9" t="inlineStr">
         <is>
@@ -920,13 +932,15 @@
       </c>
       <c r="C27" s="16" t="inlineStr"/>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>Environment: BIBS UAT environment (address issued with the passwords). Passwords: Issued separately by the iorta TechNXT Project Team; no password is written in this workbook.</t>
-        </is>
-      </c>
-    </row>
+          <t>Environment: BIBS UAT environment: https://uat.brokerverse.cloud. Passwords: Issued separately by the iorta TechNXT Project Team; no password is written in this workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
     <row r="31" ht="26" customHeight="1">
       <c r="B31" s="19" t="inlineStr">
         <is>
@@ -984,6 +998,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1383,7 +1398,7 @@
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>BIBS UAT environment (address issued with the passwords). Password: Issued separately by the iorta TechNXT Project Team</t>
+          <t>BIBS UAT environment: https://uat.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cashiering v3.2, Product Maintenance v1.2 and User Access Maintenance v1.3 rebuilt with the DEV environment address and the new screenshots; workbooks of the four packs rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_UAT_BRD-02_Business_Unit_Walkthrough_Users_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_UAT_BRD-02_Business_Unit_Walkthrough_Users_v1.0.xlsx
@@ -794,7 +794,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>10 October 2026</t>
+          <t>11 October 2026</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>BIBS UAT environment: https://uat.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
+          <t>BIBS DEV environment: https://dev.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
         </is>
       </c>
       <c r="D21" s="14" t="n">
@@ -923,7 +923,7 @@
     <row r="29">
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>Environment: BIBS UAT environment: https://uat.brokerverse.cloud. Passwords: Issued separately by the iorta TechNXT Project Team; no password is written in this workbook.</t>
+          <t>Environment: BIBS DEV environment: https://dev.brokerverse.cloud. Passwords: Issued separately by the iorta TechNXT Project Team; no password is written in this workbook.</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>BIBS UAT environment: https://uat.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
+          <t>BIBS DEV environment: https://dev.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
         </is>
       </c>
     </row>

</xml_diff>